<commit_message>
Rearranging files for change of PM
</commit_message>
<xml_diff>
--- a/BDSH - Availability.xlsx
+++ b/BDSH - Availability.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://w2shared-my.sharepoint.com/personal/dave_sushames01_student_wandw_ac_nz/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://w2shared-my.sharepoint.com/personal/dave_sushames01_student_wandw_ac_nz/Documents/Documents/Capstone/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{78D2DFD3-9ADF-4BA0-A863-344CCCDAD9B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="14" documentId="8_{78D2DFD3-9ADF-4BA0-A863-344CCCDAD9B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{59CA2E4F-0E97-4D7A-A145-4CAADB05CA93}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{5AA89B4F-44C3-4505-8EF4-0C4952A77E40}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="17">
   <si>
     <t>Mon</t>
   </si>
@@ -276,9 +276,7 @@
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="3"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="4" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="6" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="5"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="3" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="5" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
@@ -287,12 +285,14 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="6" xfId="3" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="5" xfId="3" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="6" xfId="4" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="6" xfId="5" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="5" xfId="4" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="6" xfId="6" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="1"/>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="6"/>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="6" xfId="6" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="6" xfId="5" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="7">
     <cellStyle name="20% - Accent6" xfId="5" builtinId="50"/>
@@ -637,25 +637,25 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="B1" s="9" t="s">
+      <c r="B1" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="9" t="s">
+      <c r="C1" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="9" t="s">
+      <c r="D1" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="9" t="s">
+      <c r="E1" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="9" t="s">
+      <c r="F1" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="9" t="s">
+      <c r="G1" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="H1" s="10" t="s">
+      <c r="H1" s="8" t="s">
         <v>6</v>
       </c>
       <c r="J1" s="3" t="s">
@@ -663,20 +663,20 @@
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A2" s="8">
+      <c r="A2" s="6">
         <v>9</v>
       </c>
-      <c r="C2" s="11"/>
+      <c r="C2" s="9"/>
       <c r="D2" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="E2" s="14" t="s">
+      <c r="E2" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="G2" s="17" t="s">
+      <c r="G2" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="H2" s="17" t="s">
+      <c r="H2" s="14" t="s">
         <v>12</v>
       </c>
       <c r="J2" s="2" t="s">
@@ -684,263 +684,228 @@
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A3" s="8">
+      <c r="A3" s="6">
         <v>10</v>
       </c>
-      <c r="C3" s="12"/>
+      <c r="C3" s="10"/>
       <c r="D3" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="E3" s="13" t="s">
+      <c r="E3" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="G3" s="15" t="s">
+      <c r="G3" s="13" t="s">
         <v>12</v>
       </c>
-      <c r="H3" s="15" t="s">
+      <c r="H3" s="13" t="s">
         <v>13</v>
       </c>
       <c r="J3" s="1" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A4" s="8">
-        <v>11</v>
-      </c>
-      <c r="C4" s="12"/>
+    <row r="4" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="6">
+        <v>11</v>
+      </c>
+      <c r="C4" s="10"/>
       <c r="D4" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="E4" s="13" t="s">
+      <c r="E4" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="G4" s="15" t="s">
+      <c r="G4" s="13" t="s">
         <v>12</v>
       </c>
-      <c r="H4" s="15" t="s">
+      <c r="H4" s="13" t="s">
         <v>13</v>
       </c>
       <c r="J4" s="4" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A5" s="8">
+    <row r="5" spans="1:10" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="6">
         <v>12</v>
       </c>
-      <c r="C5" s="12"/>
-      <c r="E5" s="12"/>
-      <c r="F5" s="6" t="s">
+      <c r="C5" s="10"/>
+      <c r="E5" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="F5" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="G5" s="12"/>
-      <c r="H5" s="18" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="8">
+      <c r="G5" s="10"/>
+      <c r="H5" s="15" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="6">
         <v>1</v>
       </c>
       <c r="B6" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="C6" s="12"/>
-      <c r="E6" s="15" t="s">
+      <c r="C6" s="10"/>
+      <c r="E6" s="13" t="s">
         <v>12</v>
       </c>
-      <c r="F6" s="6" t="s">
+      <c r="F6" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="G6" s="12"/>
-      <c r="H6" s="18" t="s">
+      <c r="G6" s="10"/>
+      <c r="H6" s="15" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="7" spans="1:10" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="8">
+      <c r="A7" s="6">
         <v>2</v>
       </c>
-      <c r="B7" s="21" t="s">
+      <c r="B7" s="18" t="s">
         <v>16</v>
       </c>
-      <c r="C7" s="12"/>
-      <c r="E7" s="15" t="s">
+      <c r="C7" s="10"/>
+      <c r="E7" s="13" t="s">
         <v>12</v>
       </c>
-      <c r="F7" s="6" t="s">
+      <c r="F7" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="G7" s="12"/>
-      <c r="H7" s="18" t="s">
+      <c r="G7" s="10"/>
+      <c r="H7" s="15" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="8" spans="1:10" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="8">
+      <c r="A8" s="6">
         <v>3</v>
       </c>
-      <c r="C8" s="12"/>
-      <c r="E8" s="15" t="s">
+      <c r="C8" s="10"/>
+      <c r="E8" s="13" t="s">
         <v>12</v>
       </c>
-      <c r="G8" s="12"/>
-      <c r="H8" s="18" t="s">
+      <c r="G8" s="10"/>
+      <c r="H8" s="15" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A9" s="8">
+      <c r="A9" s="6">
         <v>4</v>
       </c>
       <c r="B9" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="C9" s="13" t="s">
+      <c r="C9" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="E9" s="12"/>
-      <c r="G9" s="12"/>
-      <c r="H9" s="18" t="s">
+      <c r="E9" s="10"/>
+      <c r="G9" s="10"/>
+      <c r="H9" s="15" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A10" s="8">
+      <c r="A10" s="6">
         <v>5</v>
       </c>
-      <c r="C10" s="12"/>
-      <c r="D10" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="E10" s="16" t="s">
-        <v>11</v>
-      </c>
-      <c r="F10" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="G10" s="16" t="s">
-        <v>11</v>
-      </c>
-      <c r="H10" s="12"/>
+      <c r="C10" s="10"/>
+      <c r="E10" s="10"/>
+      <c r="F10" s="19" t="s">
+        <v>11</v>
+      </c>
+      <c r="G10" s="20" t="s">
+        <v>11</v>
+      </c>
+      <c r="H10" s="21" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A11" s="8">
+      <c r="A11" s="6">
         <v>6</v>
       </c>
-      <c r="B11" s="3" t="s">
+      <c r="C11" s="10"/>
+      <c r="E11" s="10"/>
+      <c r="F11" s="20" t="s">
+        <v>11</v>
+      </c>
+      <c r="G11" s="20" t="s">
+        <v>11</v>
+      </c>
+      <c r="H11" s="21" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A12" s="6">
+        <v>7</v>
+      </c>
+      <c r="C12" s="10"/>
+      <c r="E12" s="10"/>
+      <c r="F12" s="20" t="s">
+        <v>11</v>
+      </c>
+      <c r="G12" s="20" t="s">
+        <v>11</v>
+      </c>
+      <c r="H12" s="10"/>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A13" s="6">
+        <v>8</v>
+      </c>
+      <c r="C13" s="10"/>
+      <c r="E13" s="10"/>
+      <c r="F13" s="20" t="s">
+        <v>11</v>
+      </c>
+      <c r="G13" s="20" t="s">
+        <v>11</v>
+      </c>
+      <c r="H13" s="10"/>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A14" s="6">
+        <v>9</v>
+      </c>
+      <c r="C14" s="10"/>
+      <c r="E14" s="10"/>
+      <c r="G14" s="10"/>
+      <c r="H14" s="10"/>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A15" s="6">
+        <v>10</v>
+      </c>
+      <c r="C15" s="10"/>
+      <c r="E15" s="10"/>
+      <c r="G15" s="10"/>
+      <c r="H15" s="10"/>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A16" s="6">
+        <v>11</v>
+      </c>
+      <c r="C16" s="10"/>
+      <c r="E16" s="10"/>
+      <c r="G16" s="10"/>
+      <c r="H16" s="10"/>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A17" s="8">
         <v>12</v>
       </c>
-      <c r="C11" s="12"/>
-      <c r="D11" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="E11" s="16" t="s">
-        <v>11</v>
-      </c>
-      <c r="F11" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="G11" s="16" t="s">
-        <v>11</v>
-      </c>
-      <c r="H11" s="12"/>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A12" s="8">
-        <v>7</v>
-      </c>
-      <c r="B12" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="C12" s="12"/>
-      <c r="D12" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="E12" s="16" t="s">
-        <v>11</v>
-      </c>
-      <c r="F12" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="G12" s="16" t="s">
-        <v>11</v>
-      </c>
-      <c r="H12" s="12"/>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A13" s="8">
-        <v>8</v>
-      </c>
-      <c r="B13" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="C13" s="12"/>
-      <c r="D13" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="E13" s="16" t="s">
-        <v>11</v>
-      </c>
-      <c r="F13" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="G13" s="16" t="s">
-        <v>11</v>
-      </c>
-      <c r="H13" s="12"/>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A14" s="8">
-        <v>9</v>
-      </c>
-      <c r="B14" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="C14" s="12"/>
-      <c r="E14" s="12"/>
-      <c r="F14" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="G14" s="12"/>
-      <c r="H14" s="12"/>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A15" s="8">
-        <v>10</v>
-      </c>
-      <c r="B15" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="C15" s="12"/>
-      <c r="E15" s="12"/>
-      <c r="F15" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="G15" s="12"/>
-      <c r="H15" s="12"/>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A16" s="8">
-        <v>11</v>
-      </c>
-      <c r="C16" s="12"/>
-      <c r="E16" s="12"/>
-      <c r="G16" s="12"/>
-      <c r="H16" s="12"/>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A17" s="10">
-        <v>12</v>
-      </c>
-      <c r="B17" s="19"/>
-      <c r="C17" s="20"/>
-      <c r="D17" s="19"/>
-      <c r="E17" s="20"/>
-      <c r="F17" s="19"/>
-      <c r="G17" s="20"/>
-      <c r="H17" s="20"/>
+      <c r="B17" s="16"/>
+      <c r="C17" s="17"/>
+      <c r="D17" s="16"/>
+      <c r="E17" s="17"/>
+      <c r="F17" s="16"/>
+      <c r="G17" s="17"/>
+      <c r="H17" s="17"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>